<commit_message>
Add mana bar, Sim Results tab and first simulation script
</commit_message>
<xml_diff>
--- a/docs/Severance Design Docs.xlsx
+++ b/docs/Severance Design Docs.xlsx
@@ -15,11 +15,12 @@
     <sheet name="Base Moves" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Boss Specials" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Damage Table" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Balance Log" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Sim Results" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Balance Log" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Balance Log'!$A$4:$G$30</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Build Order'!$A$4:$H$20</definedName>
+    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Balance Log'!$A$4:$G$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Build Order'!$A$4:$H$22</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="522">
   <si>
     <t xml:space="preserve">Severance - Monster Stats</t>
   </si>
@@ -258,6 +259,9 @@
     <t xml:space="preserve">Planned (mana class)</t>
   </si>
   <si>
+    <t xml:space="preserve">Planned: Paladin Faith bar (fills when you take damage, buffs your next ability when full). See the Sim Results tab.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Paladin Abilities</t>
   </si>
   <si>
@@ -843,7 +847,7 @@
     <t xml:space="preserve">Mana bar</t>
   </si>
   <si>
-    <t xml:space="preserve">show_mana_bar in player.py, show MP cost in the menu</t>
+    <t xml:space="preserve">show_mana_bar in player.py, MP cost in the menu. Tested in a sim</t>
   </si>
   <si>
     <t xml:space="preserve">Sorcerer class + Mana Tide</t>
@@ -861,6 +865,27 @@
     <t xml:space="preserve">Tune stats + mana costs</t>
   </si>
   <si>
+    <t xml:space="preserve">Paladin Faith bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micha (mechanic) + Claude (numbers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fills when you take damage. When full, your next ability gets a power buff, then it empties. Sims on the Sim Results tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-tune enemies for Faith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All dungeons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith makes the Paladin stronger, so enemies need a small buff to keep the same difficulty</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tutorial tips per room</t>
   </si>
   <si>
@@ -870,18 +895,12 @@
     <t xml:space="preserve">XP rework: small XP from enemies, big from bosses</t>
   </si>
   <si>
-    <t xml:space="preserve">All dungeons</t>
-  </si>
-  <si>
     <t xml:space="preserve">Numbers only. Suggested split is on Dungeon Plans</t>
   </si>
   <si>
     <t xml:space="preserve">Cheetah Growl (stun)</t>
   </si>
   <si>
-    <t xml:space="preserve">Micha (mechanic) + Claude (numbers)</t>
-  </si>
-  <si>
     <t xml:space="preserve">stunned flag, Move effect, skip turn. No damage vs 0.5x hit undecided</t>
   </si>
   <si>
@@ -909,6 +928,9 @@
     <t xml:space="preserve">Micha (mechanic) + Claude (stats)</t>
   </si>
   <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
     <t xml:space="preserve">Boss adds enemies to the fight mid-battle</t>
   </si>
   <si>
@@ -927,7 +949,7 @@
     <t xml:space="preserve">Outpost</t>
   </si>
   <si>
-    <t xml:space="preserve">12</t>
+    <t xml:space="preserve">14</t>
   </si>
   <si>
     <t xml:space="preserve">Enemies/bosses drop gold, spend at a shop between dungeons (e.g. mana potions)</t>
@@ -1093,6 +1115,144 @@
   </si>
   <si>
     <t xml:space="preserve">Enraged Devastating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severance - Simulation Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each number = 4,000 simulated full runs of the dungeon (run by Claude, 1 Oct 2026). Smart = reacts to warnings and uses abilities well. Casual = uses whatever is ready, ignores warnings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea: Paladin Faith Bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Faith fills up when the Paladin takes damage (e.g. 2 Faith for every 1 HP lost, full at 100).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  When Faith is full, the next ability you use gets a power buff (more damage or more healing), then Faith empties.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Fits the tank role: the Paladin gets stronger by taking hits. Plays differently from the Sorcerer's mana.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Open questions: how big the buff is, whether Faith resets each room or carries over, and whether Defend / Divine Aegis add Faith.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status: idea only, not in the code yet. Build Order steps 6-7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 1: Should the Paladin have a bar? (Holy Strike costs from the bar, keeps its 4-turn cooldown)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rainforest Lv1 - Smart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rainforest Lv1 - Casual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spaceship Lv2 - Smart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spaceship Lv2 - Casual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Takeaway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No bar (current game)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mana 50, Holy Strike costs 10, +2 per turn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Never runs out: the bar is just decoration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mana 50, Holy Strike costs 20, +3 per turn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Much harder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mana 50, Holy Strike costs 20, +2 per turn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Far too hard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mana 40, Holy Strike costs 20, no regen, refills on rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best mana option: ~2 Holy Strikes per room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolve: fills from damage taken, Holy Strike costs 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fits a tank, hard for casual players</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolve: fills from damage taken, Holy Strike costs 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Result: Faith (below) was picked over mana and Resolve. It doesn't lock abilities, it rewards taking hits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 2: Faith bar - fills from damage taken, buffs your next ability when full</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffs per Rainforest run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffs per Spaceship run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HP left after Rainforest (smart)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 2 per HP lost, full=100, +25%, resets each room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 1 per HP lost, full=100, +25%, resets each room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 1 per HP lost, full=100, +50%, resets each room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 1 per HP lost, full=50, +50%, resets each room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 2 per HP lost, full=100, +50%, resets each room</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 2 per HP lost, full=100, +50%, kept between rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 2 per HP lost, full=100, +25%, kept between rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 2 per HP lost, full=100, +100%, kept between rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faith: 3 per HP lost, full=100, +50%, kept between rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Every Faith version makes the game easier, because it's a free buff. Bigger buff or Faith carried between rooms = easier still.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  '1 per HP lost, full at 100, resets each room' almost never fills (0.1 buffs per run), so it does nothing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Suggested start (green): 2 Faith per HP lost, full at 100, +25% buff, resets each room. About 1-2 buffs per dungeon, +5% smart / +9% casual win rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  After adding Faith, re-tune enemies slightly (Build Order step 7) to get back to the old difficulty.</t>
   </si>
   <si>
     <t xml:space="preserve">Balance Log</t>
@@ -1534,7 +1694,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1568,7 +1728,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE6E9F3"/>
-        <bgColor rgb="FFE3F1E3"/>
+        <bgColor rgb="FFEEF0F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF0F4"/>
+        <bgColor rgb="FFE6E9F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -1621,7 +1787,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1802,6 +1968,62 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1909,7 +2131,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF4D6"/>
-      <rgbColor rgb="FFE6E9F3"/>
+      <rgbColor rgb="FFEEF0F4"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1923,9 +2145,9 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFE6E9F3"/>
+      <rgbColor rgb="FFE3F1E3"/>
       <rgbColor rgb="FFF3E6E6"/>
-      <rgbColor rgb="FFE3F1E3"/>
-      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -3074,61 +3296,66 @@
         <v>74</v>
       </c>
     </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D11" s="20" t="n">
         <v>1</v>
@@ -3140,7 +3367,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H11" s="20" t="n">
         <v>0</v>
@@ -3161,18 +3388,18 @@
         <v>38</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>1</v>
@@ -3184,7 +3411,7 @@
         <v>4</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H12" s="20" t="n">
         <v>0</v>
@@ -3205,18 +3432,18 @@
         <v>58</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D13" s="20" t="n">
         <v>2</v>
@@ -3228,7 +3455,7 @@
         <v>3</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H13" s="20" t="n">
         <v>0</v>
@@ -3249,18 +3476,18 @@
         <v>38</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D14" s="20" t="n">
         <v>5</v>
@@ -3272,7 +3499,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H14" s="20" t="n">
         <v>0</v>
@@ -3293,18 +3520,18 @@
         <v>87 HP</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D15" s="20" t="n">
         <v>9</v>
@@ -3316,7 +3543,7 @@
         <v>6</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H15" s="20" t="n">
         <v>0</v>
@@ -3329,24 +3556,24 @@
         <v>18</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L15" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>13</v>
@@ -3358,7 +3585,7 @@
         <v>4</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H16" s="20" t="n">
         <v>0</v>
@@ -3379,18 +3606,18 @@
         <v>46</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D17" s="20" t="n">
         <v>20</v>
@@ -3402,7 +3629,7 @@
         <v>8</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H17" s="20" t="n">
         <v>0</v>
@@ -3423,30 +3650,30 @@
         <v>116</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>8</v>
@@ -3458,13 +3685,13 @@
         <v>11</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3496,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4128,7 +4355,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -4167,58 +4394,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>17</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4229,37 +4456,37 @@
         <v>19</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H6" s="26" t="s">
         <v>28</v>
       </c>
       <c r="I6" s="26" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L6" s="26" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="M6" s="26" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4270,37 +4497,37 @@
         <v>33</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I7" s="26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L7" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="M7" s="26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4308,40 +4535,40 @@
         <v>3</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I8" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K8" s="28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L8" s="26" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="26" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4349,13 +4576,13 @@
         <v>22</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>22</v>
@@ -4364,53 +4591,53 @@
         <v>22</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H9" s="26" t="s">
         <v>22</v>
       </c>
       <c r="I9" s="26" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K9" s="28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L9" s="26" t="s">
         <v>22</v>
       </c>
       <c r="M9" s="26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -4427,25 +4654,25 @@
         <v>19</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D13" s="26" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F13" s="26" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H13" s="26"/>
       <c r="I13" s="26"/>
       <c r="J13" s="26"/>
       <c r="K13" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4456,25 +4683,25 @@
         <v>19</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D14" s="26" t="s">
         <v>36</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H14" s="26"/>
       <c r="I14" s="26"/>
       <c r="J14" s="26"/>
       <c r="K14" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4485,25 +4712,25 @@
         <v>19</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D15" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G15" s="26" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H15" s="26"/>
       <c r="I15" s="26"/>
       <c r="J15" s="26"/>
       <c r="K15" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4517,22 +4744,22 @@
         <v>30</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E16" s="26" t="s">
         <v>28</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H16" s="26"/>
       <c r="I16" s="26"/>
       <c r="J16" s="26"/>
       <c r="K16" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4543,23 +4770,23 @@
         <v>33</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D17" s="26" t="s">
         <v>20</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G17" s="26"/>
       <c r="H17" s="26"/>
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4570,23 +4797,23 @@
         <v>33</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D18" s="26" t="s">
         <v>36</v>
       </c>
       <c r="E18" s="26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G18" s="26"/>
       <c r="H18" s="26"/>
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4597,25 +4824,25 @@
         <v>33</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D19" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E19" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="F19" s="26" t="s">
         <v>206</v>
       </c>
-      <c r="F19" s="26" t="s">
-        <v>205</v>
-      </c>
       <c r="G19" s="26" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H19" s="26"/>
       <c r="I19" s="26"/>
       <c r="J19" s="26"/>
       <c r="K19" s="29" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4626,25 +4853,25 @@
         <v>33</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D20" s="26" t="s">
         <v>30</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F20" s="26" t="s">
         <v>22</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="26"/>
       <c r="K20" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4655,25 +4882,25 @@
         <v>33</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D21" s="26" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G21" s="26" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H21" s="26"/>
       <c r="I21" s="26"/>
       <c r="J21" s="26"/>
       <c r="K21" s="27" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4684,25 +4911,25 @@
         <v>33</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D22" s="26" t="s">
         <v>30</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F22" s="26" t="s">
         <v>22</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H22" s="26"/>
       <c r="I22" s="26"/>
       <c r="J22" s="26"/>
       <c r="K22" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4710,16 +4937,16 @@
         <v>3</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D23" s="26" t="s">
         <v>5</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F23" s="26" t="s">
         <v>22</v>
@@ -4729,7 +4956,7 @@
       <c r="I23" s="26"/>
       <c r="J23" s="26"/>
       <c r="K23" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4737,28 +4964,28 @@
         <v>3</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F24" s="26" t="s">
         <v>22</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H24" s="26"/>
       <c r="I24" s="26"/>
       <c r="J24" s="26"/>
       <c r="K24" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4766,28 +4993,28 @@
         <v>3</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D25" s="26" t="s">
         <v>5</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F25" s="26" t="s">
         <v>22</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H25" s="26"/>
       <c r="I25" s="26"/>
       <c r="J25" s="26"/>
       <c r="K25" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4795,16 +5022,16 @@
         <v>3</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F26" s="26" t="s">
         <v>22</v>
@@ -4814,7 +5041,7 @@
       <c r="I26" s="26"/>
       <c r="J26" s="26"/>
       <c r="K26" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4822,28 +5049,28 @@
         <v>3</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D27" s="26" t="s">
         <v>5</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F27" s="26" t="s">
         <v>22</v>
       </c>
       <c r="G27" s="26" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H27" s="26"/>
       <c r="I27" s="26"/>
       <c r="J27" s="26"/>
       <c r="K27" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4851,93 +5078,93 @@
         <v>3</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D28" s="26" t="s">
         <v>30</v>
       </c>
       <c r="E28" s="26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F28" s="26" t="s">
         <v>22</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H28" s="26"/>
       <c r="I28" s="26"/>
       <c r="J28" s="26"/>
       <c r="K28" s="28" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="30" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="30" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="30" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="30" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="30" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="30" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="30" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="30" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4"/>
       <c r="B41" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -4953,7 +5180,7 @@
         <v>18</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D42" s="6" t="n">
         <v>5</v>
@@ -4968,7 +5195,7 @@
         <v>24</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D43" s="6" t="n">
         <v>8</v>
@@ -4983,7 +5210,7 @@
         <v>26</v>
       </c>
       <c r="C44" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D44" s="6" t="n">
         <v>12</v>
@@ -4995,10 +5222,10 @@
     <row r="45" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="26"/>
       <c r="B45" s="26" t="s">
+        <v>247</v>
+      </c>
+      <c r="C45" s="26" t="s">
         <v>246</v>
-      </c>
-      <c r="C45" s="26" t="s">
-        <v>245</v>
       </c>
       <c r="D45" s="6" t="n">
         <v>30</v>
@@ -5013,7 +5240,7 @@
         <v>32</v>
       </c>
       <c r="C46" s="26" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D46" s="6" t="n">
         <v>6</v>
@@ -5028,7 +5255,7 @@
         <v>35</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D47" s="6" t="n">
         <v>16</v>
@@ -5043,7 +5270,7 @@
         <v>37</v>
       </c>
       <c r="C48" s="26" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D48" s="6" t="n">
         <v>14</v>
@@ -5055,10 +5282,10 @@
     <row r="49" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="26"/>
       <c r="B49" s="26" t="s">
+        <v>249</v>
+      </c>
+      <c r="C49" s="26" t="s">
         <v>248</v>
-      </c>
-      <c r="C49" s="26" t="s">
-        <v>247</v>
       </c>
       <c r="D49" s="6" t="n">
         <v>45</v>
@@ -5069,7 +5296,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D50" s="31" t="n">
         <f aca="false">2*D42+3*D43+D44+D45</f>
@@ -5082,7 +5309,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D51" s="31" t="n">
         <f aca="false">2*D42+3*D43+D44</f>
@@ -5095,7 +5322,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D52" s="31" t="n">
         <f aca="false">5*D46+D47+2*D48+D49</f>
@@ -5108,7 +5335,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D53" s="31" t="n">
         <f aca="false">5*D46+D47+2*D48</f>
@@ -5121,7 +5348,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -5159,7 +5386,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -5174,32 +5401,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E4" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G4" s="32" t="s">
         <v>49</v>
@@ -5213,25 +5440,25 @@
         <v>1</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>72</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F5" s="33" t="s">
         <v>22</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5239,51 +5466,51 @@
         <v>2</v>
       </c>
       <c r="B6" s="26" t="s">
+        <v>268</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="E6" s="33" t="s">
+        <v>265</v>
+      </c>
+      <c r="F6" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="H6" s="34" t="s">
         <v>267</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>263</v>
-      </c>
-      <c r="E6" s="33" t="s">
-        <v>264</v>
-      </c>
-      <c r="F6" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="26" t="s">
-        <v>268</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C7" s="26" t="s">
         <v>72</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F7" s="33" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>270</v>
-      </c>
-      <c r="H7" s="35" t="s">
-        <v>172</v>
+        <v>271</v>
+      </c>
+      <c r="H7" s="34" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5291,25 +5518,25 @@
         <v>4</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C8" s="26" t="s">
         <v>72</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F8" s="33" t="s">
         <v>27</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H8" s="35" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5317,51 +5544,51 @@
         <v>5</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C9" s="26" t="s">
         <v>72</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>245</v>
+        <v>70</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>264</v>
+        <v>158</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="H10" s="35" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5369,51 +5596,51 @@
         <v>7</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>22</v>
+        <v>282</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="H11" s="35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F12" s="33" t="s">
         <v>22</v>
       </c>
       <c r="G12" s="26" t="s">
-        <v>283</v>
-      </c>
-      <c r="H12" s="36" t="s">
-        <v>284</v>
+        <v>285</v>
+      </c>
+      <c r="H12" s="35" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5421,16 +5648,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>163</v>
+        <v>281</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>157</v>
+        <v>265</v>
       </c>
       <c r="F13" s="33" t="s">
         <v>22</v>
@@ -5439,10 +5666,10 @@
         <v>287</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="33" t="n">
         <v>10</v>
       </c>
@@ -5450,13 +5677,13 @@
         <v>288</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>157</v>
+        <v>265</v>
       </c>
       <c r="F14" s="33" t="s">
         <v>22</v>
@@ -5464,8 +5691,8 @@
       <c r="G14" s="26" t="s">
         <v>289</v>
       </c>
-      <c r="H14" s="35" t="s">
-        <v>172</v>
+      <c r="H14" s="36" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5473,42 +5700,42 @@
         <v>11</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>247</v>
+        <v>164</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>189</v>
+        <v>22</v>
       </c>
       <c r="G15" s="26" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H15" s="35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>110</v>
+        <v>248</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>294</v>
+        <v>158</v>
       </c>
       <c r="F16" s="33" t="s">
         <v>22</v>
@@ -5517,7 +5744,7 @@
         <v>295</v>
       </c>
       <c r="H16" s="35" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5528,13 +5755,13 @@
         <v>296</v>
       </c>
       <c r="C17" s="26" t="s">
+        <v>248</v>
+      </c>
+      <c r="D17" s="26" t="s">
         <v>297</v>
       </c>
-      <c r="D17" s="26" t="s">
-        <v>263</v>
-      </c>
       <c r="E17" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F17" s="33" t="s">
         <v>298</v>
@@ -5543,7 +5770,7 @@
         <v>299</v>
       </c>
       <c r="H17" s="35" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5554,10 +5781,10 @@
         <v>300</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>297</v>
+        <v>111</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E18" s="33" t="s">
         <v>301</v>
@@ -5569,10 +5796,10 @@
         <v>302</v>
       </c>
       <c r="H18" s="35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="33" t="n">
         <v>15</v>
       </c>
@@ -5580,53 +5807,105 @@
         <v>303</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>110</v>
+        <v>304</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H19" s="35" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="33" t="n">
         <v>16</v>
       </c>
       <c r="B20" s="26" t="s">
+        <v>307</v>
+      </c>
+      <c r="C20" s="26" t="s">
+        <v>304</v>
+      </c>
+      <c r="D20" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>308</v>
+      </c>
+      <c r="F20" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="H20" s="35" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>310</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="E21" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="F21" s="33" t="s">
         <v>305</v>
       </c>
-      <c r="C20" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="D20" s="26" t="s">
-        <v>263</v>
-      </c>
-      <c r="E20" s="33" t="s">
-        <v>157</v>
-      </c>
-      <c r="F20" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="G20" s="26" t="s">
-        <v>306</v>
-      </c>
-      <c r="H20" s="35" t="s">
-        <v>172</v>
+      <c r="G21" s="26" t="s">
+        <v>311</v>
+      </c>
+      <c r="H21" s="35" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="33" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>312</v>
+      </c>
+      <c r="C22" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>264</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="F22" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" s="26" t="s">
+        <v>313</v>
+      </c>
+      <c r="H22" s="35" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H20"/>
-  <conditionalFormatting sqref="H5:H20">
+  <autoFilter ref="A4:H22"/>
+  <conditionalFormatting sqref="H5:H22">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Done"</formula>
     </cfRule>
@@ -5641,7 +5920,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H20" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H22" type="list">
       <formula1>"Done,In progress,Not started,Undecided"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5675,32 +5954,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5717,15 +5996,15 @@
         <v>1</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B6" s="37" t="n">
         <v>0.2</v>
@@ -5737,15 +6016,15 @@
         <v>0</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B7" s="37" t="n">
         <v>0.2</v>
@@ -5757,15 +6036,15 @@
         <v>1</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B8" s="37" t="n">
         <v>0.1</v>
@@ -5777,15 +6056,15 @@
         <v>0</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>22</v>
@@ -5797,15 +6076,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B11" s="39" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -5843,12 +6122,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5856,31 +6135,31 @@
         <v>30</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5916,7 +6195,7 @@
         <v>60</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5924,7 +6203,7 @@
         <v>38</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="C6" s="37" t="n">
         <v>0.2</v>
@@ -5952,7 +6231,7 @@
         <v>34</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5960,7 +6239,7 @@
         <v>38</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="C7" s="37" t="n">
         <v>0.15</v>
@@ -5988,7 +6267,7 @@
         <v>24</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6024,7 +6303,7 @@
         <v>119</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6032,7 +6311,7 @@
         <v>47</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="C9" s="37" t="n">
         <v>0.15</v>
@@ -6060,7 +6339,7 @@
         <v>189</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6068,7 +6347,7 @@
         <v>47</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="C10" s="37" t="n">
         <v>0.15</v>
@@ -6096,7 +6375,7 @@
         <v>113</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6104,7 +6383,7 @@
         <v>47</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="C11" s="37" t="n">
         <v>0.1</v>
@@ -6132,12 +6411,12 @@
         <v>88</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -6169,12 +6448,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6185,22 +6464,22 @@
         <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6657,6 +6936,553 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="45" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="46" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="47" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="48" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="48" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="48" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="48" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="46" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="47" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="49" t="s">
+        <v>376</v>
+      </c>
+      <c r="B13" s="50" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="C13" s="50" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="D13" s="50" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="E13" s="50" t="n">
+        <v>0.607</v>
+      </c>
+      <c r="F13" s="49" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="51" t="s">
+        <v>378</v>
+      </c>
+      <c r="B14" s="25" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="D14" s="25" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>0.619</v>
+      </c>
+      <c r="F14" s="51" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="51" t="s">
+        <v>380</v>
+      </c>
+      <c r="B15" s="25" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="C15" s="25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="51" t="s">
+        <v>382</v>
+      </c>
+      <c r="B16" s="25" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="C16" s="25" t="n">
+        <v>0.337</v>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="F16" s="51" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="51" t="s">
+        <v>384</v>
+      </c>
+      <c r="B17" s="25" t="n">
+        <v>0.845</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="F17" s="51" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="51" t="s">
+        <v>386</v>
+      </c>
+      <c r="B18" s="25" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="F18" s="51" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="51" t="s">
+        <v>388</v>
+      </c>
+      <c r="B19" s="25" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="F19" s="51" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="46" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="47" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="49" t="s">
+        <v>376</v>
+      </c>
+      <c r="B24" s="50" t="n">
+        <v>0.86625</v>
+      </c>
+      <c r="C24" s="50" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="D24" s="50" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="E24" s="50" t="n">
+        <v>0.614</v>
+      </c>
+      <c r="F24" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="53" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="54" t="s">
+        <v>394</v>
+      </c>
+      <c r="B25" s="55" t="n">
+        <v>0.91575</v>
+      </c>
+      <c r="C25" s="55" t="n">
+        <v>0.72775</v>
+      </c>
+      <c r="D25" s="55" t="n">
+        <v>0.9435</v>
+      </c>
+      <c r="E25" s="55" t="n">
+        <v>0.719</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G25" s="56" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H25" s="57" t="n">
+        <v>0.258333333333333</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="51" t="s">
+        <v>395</v>
+      </c>
+      <c r="B26" s="25" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="C26" s="25" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>0.92425</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>0.63175</v>
+      </c>
+      <c r="F26" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G26" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H26" s="21" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="51" t="s">
+        <v>396</v>
+      </c>
+      <c r="B27" s="25" t="n">
+        <v>0.87675</v>
+      </c>
+      <c r="C27" s="25" t="n">
+        <v>0.6865</v>
+      </c>
+      <c r="D27" s="25" t="n">
+        <v>0.9285</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>0.62375</v>
+      </c>
+      <c r="F27" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G27" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H27" s="21" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="51" t="s">
+        <v>397</v>
+      </c>
+      <c r="B28" s="25" t="n">
+        <v>0.95275</v>
+      </c>
+      <c r="C28" s="25" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="D28" s="25" t="n">
+        <v>0.9685</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>0.7745</v>
+      </c>
+      <c r="F28" s="58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G28" s="58" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H28" s="21" t="n">
+        <v>0.308333333333333</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="51" t="s">
+        <v>398</v>
+      </c>
+      <c r="B29" s="25" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C29" s="25" t="n">
+        <v>0.815</v>
+      </c>
+      <c r="D29" s="25" t="n">
+        <v>0.9635</v>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>0.78075</v>
+      </c>
+      <c r="F29" s="58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G29" s="58" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H29" s="21" t="n">
+        <v>0.304166666666667</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="51" t="s">
+        <v>399</v>
+      </c>
+      <c r="B30" s="25" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="C30" s="25" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="D30" s="25" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="E30" s="25" t="n">
+        <v>0.8535</v>
+      </c>
+      <c r="F30" s="58" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G30" s="58" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" s="21" t="n">
+        <v>0.316666666666667</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="51" t="s">
+        <v>400</v>
+      </c>
+      <c r="B31" s="25" t="n">
+        <v>0.93475</v>
+      </c>
+      <c r="C31" s="25" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="D31" s="25" t="n">
+        <v>0.9675</v>
+      </c>
+      <c r="E31" s="25" t="n">
+        <v>0.75075</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H31" s="21" t="n">
+        <v>0.266666666666667</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="51" t="s">
+        <v>401</v>
+      </c>
+      <c r="B32" s="25" t="n">
+        <v>0.98525</v>
+      </c>
+      <c r="C32" s="25" t="n">
+        <v>0.90425</v>
+      </c>
+      <c r="D32" s="25" t="n">
+        <v>0.99625</v>
+      </c>
+      <c r="E32" s="25" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="F32" s="58" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G32" s="58" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H32" s="21" t="n">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="51" t="s">
+        <v>402</v>
+      </c>
+      <c r="B33" s="25" t="n">
+        <v>0.9845</v>
+      </c>
+      <c r="C33" s="25" t="n">
+        <v>0.8385</v>
+      </c>
+      <c r="D33" s="25" t="n">
+        <v>0.98725</v>
+      </c>
+      <c r="E33" s="25" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="F33" s="58" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G33" s="58" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H33" s="21" t="n">
+        <v>0.325</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="48" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="48" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="48" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="48" t="s">
+        <v>406</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -6674,633 +7500,633 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>354</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>355</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>356</v>
+        <v>409</v>
       </c>
       <c r="B4" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>357</v>
+        <v>410</v>
       </c>
       <c r="D4" s="32" t="s">
-        <v>358</v>
+        <v>411</v>
       </c>
       <c r="E4" s="32" t="s">
-        <v>359</v>
+        <v>412</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>360</v>
+        <v>413</v>
       </c>
       <c r="G4" s="32" t="s">
-        <v>361</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>362</v>
+        <v>415</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>363</v>
+        <v>416</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>364</v>
+        <v>417</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>365</v>
+        <v>418</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>366</v>
+        <v>419</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>367</v>
+        <v>420</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>362</v>
+        <v>415</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>369</v>
+        <v>422</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>370</v>
+        <v>423</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>371</v>
+        <v>424</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>372</v>
+        <v>425</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>373</v>
+        <v>426</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>374</v>
+        <v>427</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>375</v>
+        <v>428</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>376</v>
+        <v>429</v>
       </c>
       <c r="D7" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>377</v>
+        <v>430</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>378</v>
+        <v>431</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>374</v>
+        <v>427</v>
       </c>
       <c r="B8" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>379</v>
+        <v>432</v>
       </c>
       <c r="D8" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>380</v>
+        <v>433</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>381</v>
+        <v>434</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="26" t="s">
-        <v>374</v>
+        <v>427</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>382</v>
+        <v>435</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>383</v>
+        <v>436</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>384</v>
+        <v>437</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>386</v>
+        <v>439</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>387</v>
+        <v>440</v>
       </c>
       <c r="E10" s="26" t="s">
-        <v>388</v>
+        <v>441</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>389</v>
+        <v>442</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>391</v>
+        <v>444</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>392</v>
+        <v>445</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>393</v>
+        <v>446</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>394</v>
+        <v>447</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>395</v>
+        <v>448</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>396</v>
+        <v>449</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>397</v>
+        <v>450</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>398</v>
+        <v>451</v>
       </c>
       <c r="G12" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>375</v>
+        <v>428</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>376</v>
+        <v>429</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>377</v>
+        <v>430</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>399</v>
+        <v>452</v>
       </c>
       <c r="F13" s="26" t="s">
-        <v>400</v>
+        <v>453</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>401</v>
+        <v>454</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>402</v>
+        <v>455</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>403</v>
+        <v>456</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>404</v>
+        <v>457</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>405</v>
+        <v>458</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>406</v>
+        <v>459</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>407</v>
+        <v>460</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>408</v>
+        <v>461</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>409</v>
+        <v>462</v>
       </c>
       <c r="G15" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>410</v>
+        <v>463</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>411</v>
+        <v>464</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>412</v>
+        <v>465</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>413</v>
+        <v>466</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>414</v>
+        <v>467</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>363</v>
+        <v>416</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>415</v>
+        <v>468</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>416</v>
+        <v>469</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>417</v>
+        <v>470</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>418</v>
+        <v>471</v>
       </c>
       <c r="G17" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>363</v>
+        <v>416</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>419</v>
+        <v>472</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>420</v>
+        <v>473</v>
       </c>
       <c r="E18" s="26" t="s">
-        <v>421</v>
+        <v>474</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>422</v>
+        <v>475</v>
       </c>
       <c r="G18" s="26" t="s">
-        <v>423</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>424</v>
+        <v>477</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>425</v>
+        <v>478</v>
       </c>
       <c r="E19" s="26" t="s">
-        <v>426</v>
+        <v>479</v>
       </c>
       <c r="F19" s="26" t="s">
-        <v>427</v>
+        <v>480</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>428</v>
+        <v>481</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>429</v>
+        <v>482</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>430</v>
+        <v>483</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>431</v>
+        <v>484</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>432</v>
+        <v>485</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>433</v>
+        <v>486</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>434</v>
+        <v>487</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>435</v>
+        <v>488</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>436</v>
+        <v>489</v>
       </c>
       <c r="G21" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>437</v>
+        <v>490</v>
       </c>
       <c r="D22" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>438</v>
+        <v>491</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>439</v>
+        <v>492</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B23" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>440</v>
+        <v>493</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>441</v>
+        <v>494</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>442</v>
+        <v>495</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B24" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>443</v>
+        <v>496</v>
       </c>
       <c r="D24" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>444</v>
+        <v>497</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>445</v>
+        <v>498</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B25" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>446</v>
+        <v>499</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>430</v>
+        <v>483</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>447</v>
+        <v>500</v>
       </c>
       <c r="F25" s="26" t="s">
-        <v>448</v>
+        <v>501</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B26" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>449</v>
+        <v>502</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>450</v>
+        <v>503</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>451</v>
+        <v>504</v>
       </c>
       <c r="F26" s="26" t="s">
-        <v>452</v>
+        <v>505</v>
       </c>
       <c r="G26" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>453</v>
+        <v>506</v>
       </c>
       <c r="D27" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>454</v>
+        <v>507</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G27" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>456</v>
+        <v>509</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>457</v>
+        <v>510</v>
       </c>
       <c r="D28" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E28" s="26" t="s">
-        <v>458</v>
+        <v>511</v>
       </c>
       <c r="F28" s="26" t="s">
-        <v>459</v>
+        <v>512</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="26" t="s">
-        <v>385</v>
+        <v>438</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>460</v>
+        <v>513</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>461</v>
+        <v>514</v>
       </c>
       <c r="D29" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>462</v>
+        <v>515</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>463</v>
+        <v>516</v>
       </c>
       <c r="G29" s="26" t="s">
-        <v>368</v>
+        <v>421</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="26" t="s">
-        <v>464</v>
+        <v>517</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>465</v>
+        <v>518</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>466</v>
+        <v>519</v>
       </c>
       <c r="E30" s="26" t="s">
-        <v>467</v>
+        <v>520</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>468</v>
+        <v>521</v>
       </c>
       <c r="G30" s="26" t="s">
-        <v>390</v>
+        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sorcerer: Chain Lightning 20 -> 12 MP
Sorcerer ran out of mana in the Spaceship (64%). 10 MP matched the Paladin exactly, chose 12 MP (~83%) to keep a little challenge. Rainforest unaffected.
</commit_message>
<xml_diff>
--- a/docs/Severance Design Docs.xlsx
+++ b/docs/Severance Design Docs.xlsx
@@ -19,7 +19,7 @@
     <sheet name="Balance Log" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Balance Log'!$A$4:$G$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Balance Log'!$A$4:$G$33</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Build Order'!$A$4:$H$24</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="599">
   <si>
     <t xml:space="preserve">Severance - Monster Stats</t>
   </si>
@@ -949,7 +949,7 @@
     <t xml:space="preserve">Smarter sim bot</t>
   </si>
   <si>
-    <t xml:space="preserve">Use AOE when 2+ enemies, strongest ability first. Current bot uses abilities in menu order, so Spaceship numbers are low</t>
+    <t xml:space="preserve">AOE when 2+ enemies, strongest ability first, heals below half HP, Mana Tide only when nothing else is ready. Paladin Spaceship 48% -&gt; 86%</t>
   </si>
   <si>
     <t xml:space="preserve">Paladin Faith bar</t>
@@ -1399,6 +1399,57 @@
     <t xml:space="preserve">Spaceship at Lv 2 with the same bot: Paladin 48%, Sorcerer 61%. Low for both because the bot uses abilities in menu order (no AOE priority) - see Build Order step 7.</t>
   </si>
   <si>
+    <t xml:space="preserve">Test 4: Sorcerer mana in the Spaceship (smarter bot: AOE first, best ability, Mana Tide on off-turns; 5,000-8,000 runs each)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorcerer before (regen 4, Chain Lightning 20 MP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs out of mana against groups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mana regen 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Makes the Rainforest too easy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mana regen 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max mana 80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fire Bolt 8 MP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain Lightning 15 MP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only changes the Spaceship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain Lightning 12 MP (chosen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slightly harder than the Paladin on purpose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain Lightning 10 MP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches the Paladin exactly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain Lightning 15 MP, 1.3x power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  Changing regen or max mana affects every fight from Lv 1, so the Rainforest gets too easy. Chain Lightning unlocks at Lv 2 (after the Rainforest boss), so it only changes the Spaceship.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  10 MP would have matched the Paladin exactly, but we picked 12 MP to keep a little bit of a challenge for the Sorcerer.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Balance Log</t>
   </si>
   <si>
@@ -1766,6 +1817,18 @@
   </si>
   <si>
     <t xml:space="preserve">Simulation (Micha's simulate.py)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain Lightning mana cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 MP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 MP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorcerer ran out of mana in the Spaceship (64% vs Paladin 86%). 10 MP would have matched the Paladin exactly (86%), but we went with 12 (83%) to keep a little bit of a challenge. Rainforest unaffected (unlocks at Lv 2)</t>
   </si>
 </sst>
 </file>
@@ -1956,7 +2019,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2187,6 +2250,10 @@
     </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -4676,7 +4743,7 @@
         <v>101</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="I50" s="26" t="s">
         <v>22</v>
@@ -6602,27 +6669,27 @@
   <dimension ref="A1:H24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="21" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
         <v>280</v>
       </c>
@@ -6648,7 +6715,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="37" t="n">
         <v>1</v>
       </c>
@@ -6674,7 +6741,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="37" t="n">
         <v>2</v>
       </c>
@@ -6700,7 +6767,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37" t="n">
         <v>3</v>
       </c>
@@ -6726,7 +6793,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37" t="n">
         <v>4</v>
       </c>
@@ -6752,7 +6819,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="37" t="n">
         <v>5</v>
       </c>
@@ -6778,7 +6845,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="37" t="n">
         <v>6</v>
       </c>
@@ -6804,7 +6871,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="37" t="n">
         <v>7</v>
       </c>
@@ -6815,7 +6882,7 @@
         <v>111</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>288</v>
@@ -6826,11 +6893,11 @@
       <c r="G11" s="30" t="s">
         <v>305</v>
       </c>
-      <c r="H11" s="39" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="H11" s="38" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="37" t="n">
         <v>8</v>
       </c>
@@ -6856,7 +6923,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="37" t="n">
         <v>9</v>
       </c>
@@ -6882,7 +6949,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="37" t="n">
         <v>10</v>
       </c>
@@ -6908,7 +6975,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="37" t="n">
         <v>11</v>
       </c>
@@ -6934,7 +7001,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="37" t="n">
         <v>12</v>
       </c>
@@ -6960,7 +7027,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="37" t="n">
         <v>13</v>
       </c>
@@ -6986,7 +7053,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="37" t="n">
         <v>14</v>
       </c>
@@ -7012,7 +7079,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="37" t="n">
         <v>15</v>
       </c>
@@ -7038,7 +7105,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="37" t="n">
         <v>16</v>
       </c>
@@ -7064,7 +7131,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="37" t="n">
         <v>17</v>
       </c>
@@ -7090,7 +7157,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="37" t="n">
         <v>18</v>
       </c>
@@ -7116,7 +7183,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="37" t="n">
         <v>19</v>
       </c>
@@ -7142,7 +7209,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="37" t="n">
         <v>20</v>
       </c>
@@ -8205,7 +8272,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
@@ -8892,6 +8959,175 @@
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
         <v>454</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="22" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="49" t="s">
+        <v>438</v>
+      </c>
+      <c r="B57" s="50" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="C57" s="50" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="D57" s="49" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="23" t="s">
+        <v>456</v>
+      </c>
+      <c r="B58" s="29" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="C58" s="29" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="D58" s="23" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="23" t="s">
+        <v>458</v>
+      </c>
+      <c r="B59" s="29" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="C59" s="29" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="D59" s="23" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="23" t="s">
+        <v>460</v>
+      </c>
+      <c r="B60" s="29" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="C60" s="29" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="D60" s="23" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="23" t="s">
+        <v>461</v>
+      </c>
+      <c r="B61" s="29" t="n">
+        <v>0.948</v>
+      </c>
+      <c r="C61" s="29" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="D61" s="23" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="23" t="s">
+        <v>462</v>
+      </c>
+      <c r="B62" s="29" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="C62" s="29" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D62" s="23" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="B63" s="29" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="C63" s="29" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="D63" s="23" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="53" t="s">
+        <v>465</v>
+      </c>
+      <c r="B64" s="54" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="C64" s="54" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="D64" s="53" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="23" t="s">
+        <v>467</v>
+      </c>
+      <c r="B65" s="29" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="C65" s="29" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="D65" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="23" t="s">
+        <v>469</v>
+      </c>
+      <c r="B66" s="29" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="C66" s="29" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="D66" s="23" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="58" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="58" t="s">
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -8910,7 +9146,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12"/>
@@ -8923,683 +9159,706 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>455</v>
+        <v>472</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>456</v>
+        <v>473</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>457</v>
+        <v>474</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>282</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>458</v>
+        <v>475</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>459</v>
+        <v>476</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>460</v>
+        <v>477</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>461</v>
+        <v>478</v>
       </c>
       <c r="G4" s="36" t="s">
-        <v>462</v>
+        <v>479</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>463</v>
+        <v>480</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>464</v>
+        <v>481</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>465</v>
+        <v>482</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>466</v>
+        <v>483</v>
       </c>
       <c r="E5" s="30" t="s">
-        <v>467</v>
+        <v>484</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>468</v>
+        <v>485</v>
       </c>
       <c r="G5" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="s">
-        <v>463</v>
+        <v>480</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>470</v>
+        <v>487</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>471</v>
+        <v>488</v>
       </c>
       <c r="E6" s="30" t="s">
-        <v>472</v>
+        <v>489</v>
       </c>
       <c r="F6" s="30" t="s">
-        <v>473</v>
+        <v>490</v>
       </c>
       <c r="G6" s="30" t="s">
-        <v>474</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
-        <v>475</v>
+        <v>492</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>476</v>
+        <v>493</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>477</v>
+        <v>494</v>
       </c>
       <c r="D7" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>478</v>
+        <v>495</v>
       </c>
       <c r="F7" s="30" t="s">
-        <v>479</v>
+        <v>496</v>
       </c>
       <c r="G7" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="s">
-        <v>475</v>
+        <v>492</v>
       </c>
       <c r="B8" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>480</v>
+        <v>497</v>
       </c>
       <c r="D8" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="30" t="s">
-        <v>481</v>
+        <v>498</v>
       </c>
       <c r="F8" s="30" t="s">
-        <v>482</v>
+        <v>499</v>
       </c>
       <c r="G8" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="s">
-        <v>475</v>
+        <v>492</v>
       </c>
       <c r="B9" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>483</v>
+        <v>500</v>
       </c>
       <c r="D9" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>484</v>
+        <v>501</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>485</v>
+        <v>502</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B10" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>487</v>
+        <v>504</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>488</v>
+        <v>505</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="F10" s="30" t="s">
-        <v>490</v>
+        <v>507</v>
       </c>
       <c r="G10" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B11" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>492</v>
+        <v>509</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>493</v>
+        <v>510</v>
       </c>
       <c r="E11" s="30" t="s">
-        <v>494</v>
+        <v>511</v>
       </c>
       <c r="F11" s="30" t="s">
-        <v>495</v>
+        <v>512</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B12" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>496</v>
+        <v>513</v>
       </c>
       <c r="D12" s="30" t="s">
-        <v>497</v>
+        <v>514</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>498</v>
+        <v>515</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>499</v>
+        <v>516</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>476</v>
+        <v>493</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>477</v>
+        <v>494</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>478</v>
+        <v>495</v>
       </c>
       <c r="E13" s="30" t="s">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="F13" s="30" t="s">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="G13" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>503</v>
+        <v>520</v>
       </c>
       <c r="D14" s="30" t="s">
-        <v>504</v>
+        <v>521</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>506</v>
+        <v>523</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B15" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C15" s="30" t="s">
-        <v>507</v>
+        <v>524</v>
       </c>
       <c r="D15" s="30" t="s">
+        <v>525</v>
+      </c>
+      <c r="E15" s="30" t="s">
+        <v>526</v>
+      </c>
+      <c r="F15" s="30" t="s">
+        <v>527</v>
+      </c>
+      <c r="G15" s="30" t="s">
         <v>508</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>509</v>
-      </c>
-      <c r="F15" s="30" t="s">
-        <v>510</v>
-      </c>
-      <c r="G15" s="30" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B16" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>511</v>
+        <v>528</v>
       </c>
       <c r="D16" s="30" t="s">
-        <v>512</v>
+        <v>529</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>513</v>
+        <v>530</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>514</v>
+        <v>531</v>
       </c>
       <c r="G16" s="30" t="s">
-        <v>515</v>
+        <v>532</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>464</v>
+        <v>481</v>
       </c>
       <c r="C17" s="30" t="s">
-        <v>516</v>
+        <v>533</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>517</v>
+        <v>534</v>
       </c>
       <c r="E17" s="30" t="s">
-        <v>518</v>
+        <v>535</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="G17" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>464</v>
+        <v>481</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>520</v>
+        <v>537</v>
       </c>
       <c r="D18" s="30" t="s">
-        <v>521</v>
+        <v>538</v>
       </c>
       <c r="E18" s="30" t="s">
-        <v>522</v>
+        <v>539</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>523</v>
+        <v>540</v>
       </c>
       <c r="G18" s="30" t="s">
-        <v>524</v>
+        <v>541</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B19" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>525</v>
+        <v>542</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>526</v>
+        <v>543</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>527</v>
+        <v>544</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>528</v>
+        <v>545</v>
       </c>
       <c r="G19" s="30" t="s">
-        <v>529</v>
+        <v>546</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B20" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>530</v>
+        <v>547</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>531</v>
+        <v>548</v>
       </c>
       <c r="E20" s="30" t="s">
-        <v>532</v>
+        <v>549</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>533</v>
+        <v>550</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B21" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>534</v>
+        <v>551</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>535</v>
+        <v>552</v>
       </c>
       <c r="E21" s="30" t="s">
-        <v>536</v>
+        <v>553</v>
       </c>
       <c r="F21" s="30" t="s">
-        <v>537</v>
+        <v>554</v>
       </c>
       <c r="G21" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B22" s="30" t="s">
         <v>208</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>538</v>
+        <v>555</v>
       </c>
       <c r="D22" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>540</v>
+        <v>557</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B23" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>541</v>
+        <v>558</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>542</v>
+        <v>559</v>
       </c>
       <c r="E23" s="30" t="s">
         <v>220</v>
       </c>
       <c r="F23" s="30" t="s">
-        <v>543</v>
+        <v>560</v>
       </c>
       <c r="G23" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B24" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>544</v>
+        <v>561</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>545</v>
+        <v>562</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>546</v>
+        <v>563</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B25" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>547</v>
+        <v>564</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>531</v>
+        <v>548</v>
       </c>
       <c r="E25" s="30" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="F25" s="30" t="s">
-        <v>549</v>
+        <v>566</v>
       </c>
       <c r="G25" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B26" s="30" t="s">
         <v>70</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>551</v>
+        <v>568</v>
       </c>
       <c r="E26" s="30" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>553</v>
+        <v>570</v>
       </c>
       <c r="G26" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B27" s="30" t="s">
         <v>271</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>554</v>
+        <v>571</v>
       </c>
       <c r="D27" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>555</v>
+        <v>572</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>556</v>
+        <v>573</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>558</v>
+        <v>575</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>559</v>
+        <v>576</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>560</v>
+        <v>577</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>561</v>
+        <v>578</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>562</v>
+        <v>579</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>563</v>
+        <v>580</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>564</v>
+        <v>581</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="30" t="s">
-        <v>565</v>
+        <v>582</v>
       </c>
       <c r="B30" s="30" t="s">
         <v>269</v>
       </c>
       <c r="C30" s="30" t="s">
-        <v>566</v>
+        <v>583</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>567</v>
+        <v>584</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="F30" s="30" t="s">
-        <v>569</v>
+        <v>586</v>
       </c>
       <c r="G30" s="30" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="30" t="s">
-        <v>565</v>
+        <v>582</v>
       </c>
       <c r="B31" s="30" t="s">
         <v>72</v>
       </c>
       <c r="C31" s="30" t="s">
-        <v>570</v>
+        <v>587</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>22</v>
       </c>
       <c r="E31" s="30" t="s">
-        <v>571</v>
+        <v>588</v>
       </c>
       <c r="F31" s="30" t="s">
-        <v>572</v>
+        <v>589</v>
       </c>
       <c r="G31" s="30" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="30" t="s">
-        <v>565</v>
+        <v>582</v>
       </c>
       <c r="B32" s="30" t="s">
         <v>72</v>
       </c>
       <c r="C32" s="30" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>574</v>
+        <v>591</v>
       </c>
       <c r="E32" s="30" t="s">
-        <v>575</v>
+        <v>592</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="G32" s="30" t="s">
-        <v>577</v>
+        <v>594</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="30" t="s">
+        <v>582</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" s="30" t="s">
+        <v>595</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>596</v>
+      </c>
+      <c r="E33" s="30" t="s">
+        <v>597</v>
+      </c>
+      <c r="F33" s="30" t="s">
+        <v>598</v>
+      </c>
+      <c r="G33" s="30" t="s">
+        <v>594</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G32"/>
+  <autoFilter ref="A4:G33"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>